<commit_message>
Update PRESS-CMS to 1020 final version
- AI interview draft panel and edge function updates
- Add dev-log for 2026-10-19 ~ 10-25, refresh deliverables
- Reorganize docs: editorial/permission docs moved to docs/guides
- Move internal docs to docs/internal (gitignored), drop metadata.json

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N4QxT81b63qrdYtJeNQiAr
</commit_message>
<xml_diff>
--- a/docs/deliverables/PRESS-CMS_요구사항분석표_테스트데이터셋.xlsx
+++ b/docs/deliverables/PRESS-CMS_요구사항분석표_테스트데이터셋.xlsx
@@ -549,7 +549,7 @@
     <t xml:space="preserve">※ 시험 자료는 모두 가상의 내용입니다(가나시, 인물 이름 포함). 실제 기사나 실존 인물과 무관합니다.</t>
   </si>
   <si>
-    <t xml:space="preserve">※ 구현 상태와 판정은 2026-10-16 기준입니다. AI 이미지(T33·T34)는 결제가 연결된 키가 있어야 시험할 수 있고, OpenAI·구글 클라우드 받아쓰기는 키가 없어 시험 전입니다.</t>
+    <t xml:space="preserve">※ 구현 상태와 판정은 2026-10-19 기준입니다. 구글 클라우드 받아쓰기(T42·T43·T46·T47)는 키 생성이 막혀 보류, T24는 실제 혼잡 때 확인 예정입니다.</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -1329,7 +1329,7 @@
     <t xml:space="preserve">T05, T10, T11, T15, T20</t>
   </si>
   <si>
-    <t xml:space="preserve">T20 부분 통과(10-14): 근거 없는 발언을 넣어 달라는 요청에 거절하지 않고 문장을 추가함([확인 필요] 표시는 붙음, 지어낸 인용문은 없음). 수정 지시문 강화 여부 결정 필요.</t>
+    <t xml:space="preserve">T20: 10-14 부분 통과 → 지시문·서버 수정 후 10-19 배포 사이트에서 통과(근거 없는 발언 요청을 넣지 않고 안내). T05·T10·T11·T15 통과.</t>
   </si>
   <si>
     <t xml:space="preserve">R-14</t>
@@ -5145,49 +5145,15 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">AI</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">가 거절하지 않고 요청한 내용의 문장을 추가함</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Malgun Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. [</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">확인 필요</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Malgun Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">] </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">표시는 붙었고 지어낸 인용문</t>
+      <t xml:space="preserve">10-14 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">부분 통과</t>
     </r>
     <r>
       <rPr>
@@ -5204,69 +5170,205 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">따옴표 발언</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Malgun Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">은 없음</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Malgun Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2026-10-14 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">로컬</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Malgun Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">부분 통과 — 수정 지시문 강화 여부 팀 결정 필요 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Malgun Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ 10-16 </t>
+      <t xml:space="preserve">문장 추가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지시문</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">서버 수정 후 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10-19 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">배포 사이트 재시험</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">본문에 환영 발언 없음</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대화창에 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">다음 요청은 취재 자료에 근거가 없어 넣지 않았습니다…사실을 확인하셨다면 답변으로 알려 주세요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">안내</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026-10-19 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">배포 사이트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(Render), gemini-3.6-flash. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">안내에 내부 용어</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(draft_state)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가 섞여 쉬운 말로 쓰게 고침</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">재배포 필요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) / 10-16 </t>
     </r>
     <r>
       <rPr>
@@ -8557,7 +8659,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -8585,14 +8687,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC8E6C9"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFE0B2"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -8923,7 +9017,7 @@
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">COUNTIF('요구사항 분석표'!$E$2:$E$15,A6)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8932,7 +9026,7 @@
       </c>
       <c r="B7" s="7" t="n">
         <f aca="false">COUNTIF('요구사항 분석표'!$E$2:$E$15,A7)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8967,7 +9061,7 @@
       </c>
       <c r="B12" s="7" t="n">
         <f aca="false">COUNTIF('테스트 데이터셋'!$I$2:$I$49,A12)</f>
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8985,7 +9079,7 @@
       </c>
       <c r="B14" s="7" t="n">
         <f aca="false">COUNTIF('테스트 데이터셋'!$I$2:$I$49,A14)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9434,7 +9528,7 @@
         <v>102</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F14" s="13" t="s">
         <v>103</v>
@@ -9473,13 +9567,13 @@
   </sheetData>
   <autoFilter ref="A1:H15"/>
   <conditionalFormatting sqref="E2:E15">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>"완료"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>"부분"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"미구현"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10155,7 +10249,7 @@
         <v>231</v>
       </c>
       <c r="I21" s="17" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J21" s="18" t="s">
         <v>232</v>
@@ -11006,10 +11100,10 @@
   </sheetData>
   <autoFilter ref="A1:J49"/>
   <conditionalFormatting sqref="I2:I49">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>"통과"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"실패"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>